<commit_message>
Age Groups: Add Basic and Adaptive templates
</commit_message>
<xml_diff>
--- a/local/agegroups/USAW.xlsx
+++ b/local/agegroups/USAW.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/agegroups/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246311FE-6F9C-3D49-B4A0-75E0BB97ECF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5D608C-8DB5-5D4D-9B2C-38A9561C465A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36840" yWindow="3160" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4540,7 +4540,8 @@
         <v>11</v>
       </c>
       <c r="F69" s="5" t="b">
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G69" s="2">
         <v>32</v>
@@ -4596,8 +4597,8 @@
         <v>13</v>
       </c>
       <c r="F70" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G70" s="2">
         <v>32</v>
@@ -4653,8 +4654,8 @@
         <v>15</v>
       </c>
       <c r="F71" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H71" s="1"/>
       <c r="I71"/>
@@ -4707,8 +4708,8 @@
         <v>17</v>
       </c>
       <c r="F72" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H72"/>
       <c r="I72"/>
@@ -4809,8 +4810,8 @@
         <v>20</v>
       </c>
       <c r="F74" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H74"/>
       <c r="I74"/>
@@ -4860,8 +4861,8 @@
         <v>999</v>
       </c>
       <c r="F75" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H75"/>
       <c r="I75"/>
@@ -6691,7 +6692,8 @@
         <v>11</v>
       </c>
       <c r="F111" s="5" t="b">
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G111" s="2">
         <v>32</v>
@@ -6747,8 +6749,8 @@
         <v>13</v>
       </c>
       <c r="F112" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G112" s="2">
         <v>32</v>
@@ -6804,8 +6806,8 @@
         <v>15</v>
       </c>
       <c r="F113" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H113" s="1"/>
       <c r="I113"/>
@@ -6858,8 +6860,8 @@
         <v>17</v>
       </c>
       <c r="F114" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H114"/>
       <c r="I114"/>
@@ -6960,8 +6962,8 @@
         <v>20</v>
       </c>
       <c r="F116" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H116"/>
       <c r="I116"/>
@@ -7011,8 +7013,8 @@
         <v>999</v>
       </c>
       <c r="F117" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H117"/>
       <c r="I117"/>
@@ -8842,7 +8844,8 @@
         <v>11</v>
       </c>
       <c r="F153" s="5" t="b">
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G153" s="2">
         <v>32</v>
@@ -8898,8 +8901,8 @@
         <v>13</v>
       </c>
       <c r="F154" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G154" s="2">
         <v>32</v>
@@ -8955,8 +8958,8 @@
         <v>15</v>
       </c>
       <c r="F155" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H155" s="1"/>
       <c r="I155"/>
@@ -9009,8 +9012,8 @@
         <v>17</v>
       </c>
       <c r="F156" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H156"/>
       <c r="I156"/>
@@ -9111,8 +9114,8 @@
         <v>20</v>
       </c>
       <c r="F158" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H158"/>
       <c r="I158"/>
@@ -9162,8 +9165,8 @@
         <v>999</v>
       </c>
       <c r="F159" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H159"/>
       <c r="I159"/>
@@ -10993,7 +10996,8 @@
         <v>11</v>
       </c>
       <c r="F195" s="5" t="b">
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G195" s="2">
         <v>32</v>
@@ -11049,8 +11053,8 @@
         <v>13</v>
       </c>
       <c r="F196" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="G196" s="2">
         <v>32</v>
@@ -11106,8 +11110,8 @@
         <v>15</v>
       </c>
       <c r="F197" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H197" s="1"/>
       <c r="I197"/>
@@ -11160,8 +11164,8 @@
         <v>17</v>
       </c>
       <c r="F198" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H198"/>
       <c r="I198"/>
@@ -11262,8 +11266,8 @@
         <v>20</v>
       </c>
       <c r="F200" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H200"/>
       <c r="I200"/>
@@ -11313,8 +11317,8 @@
         <v>999</v>
       </c>
       <c r="F201" s="5" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H201"/>
       <c r="I201"/>

</xml_diff>